<commit_message>
Pattern Pool Score Calibration
</commit_message>
<xml_diff>
--- a/assets/data/DLT历史数据_适配模型版.xlsx
+++ b/assets/data/DLT历史数据_适配模型版.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2883"/>
+  <dimension ref="A1:H2885"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75402,6 +75402,58 @@
         <v>7</v>
       </c>
     </row>
+    <row r="2884">
+      <c r="A2884" t="n">
+        <v>26065</v>
+      </c>
+      <c r="B2884" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2884" t="n">
+        <v>11</v>
+      </c>
+      <c r="D2884" t="n">
+        <v>12</v>
+      </c>
+      <c r="E2884" t="n">
+        <v>13</v>
+      </c>
+      <c r="F2884" t="n">
+        <v>25</v>
+      </c>
+      <c r="G2884" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2884" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2885">
+      <c r="A2885" t="n">
+        <v>26066</v>
+      </c>
+      <c r="B2885" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2885" t="n">
+        <v>13</v>
+      </c>
+      <c r="D2885" t="n">
+        <v>19</v>
+      </c>
+      <c r="E2885" t="n">
+        <v>21</v>
+      </c>
+      <c r="F2885" t="n">
+        <v>30</v>
+      </c>
+      <c r="G2885" t="n">
+        <v>4</v>
+      </c>
+      <c r="H2885" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>

<commit_message>
后区全枚举 C (12,2)=66 组合 + K-Medoids 覆盖优化
</commit_message>
<xml_diff>
--- a/assets/data/DLT历史数据_适配模型版.xlsx
+++ b/assets/data/DLT历史数据_适配模型版.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2888"/>
+  <dimension ref="A1:H2889"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75532,6 +75532,32 @@
         <v>10</v>
       </c>
     </row>
+    <row r="2889">
+      <c r="A2889" t="n">
+        <v>26070</v>
+      </c>
+      <c r="B2889" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2889" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2889" t="n">
+        <v>15</v>
+      </c>
+      <c r="E2889" t="n">
+        <v>21</v>
+      </c>
+      <c r="F2889" t="n">
+        <v>32</v>
+      </c>
+      <c r="G2889" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2889" t="n">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>

</xml_diff>